<commit_message>
Updated with new form fields
</commit_message>
<xml_diff>
--- a/public/csvdata/variablenamelookups.xlsx
+++ b/public/csvdata/variablenamelookups.xlsx
@@ -1,22 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidhochbaum/ae-cd-needs-statements-generator/public/csvdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90A33F6A-53FD-4042-9057-9786AF044171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D6ECA8-101D-9B4A-99B0-3BB1AF96C8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49160" yWindow="-4280" windowWidth="26440" windowHeight="15440" activeTab="1" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
+    <workbookView xWindow="49160" yWindow="-4300" windowWidth="26440" windowHeight="15440" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Statements" sheetId="1" r:id="rId1"/>
     <sheet name="brs" sheetId="2" r:id="rId2"/>
+    <sheet name="Agency Acronyms" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">brs!$A$1:$B$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Statements!$A$1:$B$146</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="304">
   <si>
     <t>Response ID</t>
   </si>
@@ -135,12 +140,6 @@
     <t>Done!:Progress Tracking Check this box when you've completed this page.</t>
   </si>
   <si>
-    <t>communityDistrictOverview</t>
-  </si>
-  <si>
-    <t>Your FY25 Community District Overview</t>
-  </si>
-  <si>
     <t>1:Please use the this File Upload button if you would like to attach any additional files to this section of the report.¬†</t>
   </si>
   <si>
@@ -573,36 +572,6 @@
     <t>Is this request specific to a particular site, location, or facility?</t>
   </si>
   <si>
-    <t>siteAddress</t>
-  </si>
-  <si>
-    <t>Address:Request Location (complete all that apply)</t>
-  </si>
-  <si>
-    <t>siteSiteName</t>
-  </si>
-  <si>
-    <t>Site Name:Request Location (complete all that apply)</t>
-  </si>
-  <si>
-    <t>siteFacilityName</t>
-  </si>
-  <si>
-    <t>Facility Name:Request Location (complete all that apply)</t>
-  </si>
-  <si>
-    <t>siteCrossStreet1</t>
-  </si>
-  <si>
-    <t>Cross-Street 1 (for Street Segment):Request Location (complete all that apply)</t>
-  </si>
-  <si>
-    <t>siteCrossStreet2</t>
-  </si>
-  <si>
-    <t>Cross-Street 2 (for Street Segment):Request Location (complete all that apply)</t>
-  </si>
-  <si>
     <t>address-search.js</t>
   </si>
   <si>
@@ -703,23 +672,298 @@
   </si>
   <si>
     <t>agencyAcronym</t>
+  </si>
+  <si>
+    <t>Access Log</t>
+  </si>
+  <si>
+    <t>Address:Request Location (complete all that apply) For addresses, please select an option from the Address Search drop down where possible.</t>
+  </si>
+  <si>
+    <t>Site or Facility Name:Request Location (complete all that apply) For addresses, please select an option from the Address Search drop down where possible.</t>
+  </si>
+  <si>
+    <t>Facility Name:Request Location (complete all that apply) For addresses, please select an option from the Address Search drop down where possible.</t>
+  </si>
+  <si>
+    <t>Cross-Street 1 (for Street Segment):Request Location (complete all that apply) For addresses, please select an option from the Address Search drop down where possible.</t>
+  </si>
+  <si>
+    <t>Cross-Street 2 (for Street Segment):Request Location (complete all that apply) For addresses, please select an option from the Address Search drop down where possible.</t>
+  </si>
+  <si>
+    <t>Supporter 1</t>
+  </si>
+  <si>
+    <t>Supporter 2</t>
+  </si>
+  <si>
+    <t>Previous Year ID</t>
+  </si>
+  <si>
+    <t>Current Year ID</t>
+  </si>
+  <si>
+    <t>supporter1</t>
+  </si>
+  <si>
+    <t>supporter2</t>
+  </si>
+  <si>
+    <t>currentYearID</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>siteOrFacility</t>
+  </si>
+  <si>
+    <t>DPR</t>
+  </si>
+  <si>
+    <t>HRA</t>
+  </si>
+  <si>
+    <t>DCLA</t>
+  </si>
+  <si>
+    <t>DOT</t>
+  </si>
+  <si>
+    <t>DFTA</t>
+  </si>
+  <si>
+    <t>NYPD</t>
+  </si>
+  <si>
+    <t>LPC</t>
+  </si>
+  <si>
+    <t>DOE</t>
+  </si>
+  <si>
+    <t>DSNY</t>
+  </si>
+  <si>
+    <t>NYCTA</t>
+  </si>
+  <si>
+    <t>DHS</t>
+  </si>
+  <si>
+    <t>DCP</t>
+  </si>
+  <si>
+    <t>DEP</t>
+  </si>
+  <si>
+    <t>DOHMH</t>
+  </si>
+  <si>
+    <t>FDNY</t>
+  </si>
+  <si>
+    <t>HHC</t>
+  </si>
+  <si>
+    <t>HPD</t>
+  </si>
+  <si>
+    <t>NYCHA</t>
+  </si>
+  <si>
+    <t>NYCEM</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>SBS</t>
+  </si>
+  <si>
+    <t>DCAS</t>
+  </si>
+  <si>
+    <t>SCA</t>
+  </si>
+  <si>
+    <t>DYCD</t>
+  </si>
+  <si>
+    <t>ACS</t>
+  </si>
+  <si>
+    <t>NYPL</t>
+  </si>
+  <si>
+    <t>BPL</t>
+  </si>
+  <si>
+    <t>QL</t>
+  </si>
+  <si>
+    <t>OMB</t>
+  </si>
+  <si>
+    <t>TLC</t>
+  </si>
+  <si>
+    <t>MOME</t>
+  </si>
+  <si>
+    <t>MOCJ</t>
+  </si>
+  <si>
+    <t>EDC</t>
+  </si>
+  <si>
+    <t>DOITT</t>
+  </si>
+  <si>
+    <t>DOB</t>
+  </si>
+  <si>
+    <t>DCWP</t>
+  </si>
+  <si>
+    <t>Department of Parks and Recreation (DPR)</t>
+  </si>
+  <si>
+    <t>Human Resources Administration (HRA)</t>
+  </si>
+  <si>
+    <t>Department of Cultural Affairs (DCLA)</t>
+  </si>
+  <si>
+    <t>Department of Transportation (DOT)</t>
+  </si>
+  <si>
+    <t>Department for the Aging (DFTA)</t>
+  </si>
+  <si>
+    <t>New York Police Department (NYPD)</t>
+  </si>
+  <si>
+    <t>Landmarks Preservation Commission (LPC)</t>
+  </si>
+  <si>
+    <t>Department of Education (DOE)</t>
+  </si>
+  <si>
+    <t>Department of Sanitation (DSNY)</t>
+  </si>
+  <si>
+    <t>New York City Transit Authority (NYCTA)</t>
+  </si>
+  <si>
+    <t>Department for Homeless Services (DHS)</t>
+  </si>
+  <si>
+    <t>Department of City Planning (DCP)</t>
+  </si>
+  <si>
+    <t>Department of Environmental Protection (DEP)</t>
+  </si>
+  <si>
+    <t>Department of Health and Mental Hygiene (DOHMH)</t>
+  </si>
+  <si>
+    <t>Fire Department of New York (FDNY)</t>
+  </si>
+  <si>
+    <t>Health and Hospitals Corporation (HHC)</t>
+  </si>
+  <si>
+    <t>Housing Preservation and Development (HPD)</t>
+  </si>
+  <si>
+    <t>New York City Housing Authority (NYCHA)</t>
+  </si>
+  <si>
+    <t>NYC Emergency Management (NYCEM)</t>
+  </si>
+  <si>
+    <t>Department of Small Business Services (SBS)</t>
+  </si>
+  <si>
+    <t>Department of Citywide Administrative Services (DCAS)</t>
+  </si>
+  <si>
+    <t>School Construction Authority</t>
+  </si>
+  <si>
+    <t>Department of Youth and Community Development (DYCD)</t>
+  </si>
+  <si>
+    <t>Administration for Children's Services (ACS)</t>
+  </si>
+  <si>
+    <t>New York Public Library (NYPL)</t>
+  </si>
+  <si>
+    <t>Brooklyn Public Library (BPL)</t>
+  </si>
+  <si>
+    <t>Queens Library (QL)</t>
+  </si>
+  <si>
+    <t>Office of Management and Budget (OMB)</t>
+  </si>
+  <si>
+    <t>Taxi and Limousine Commission (TLC)</t>
+  </si>
+  <si>
+    <t>Mayor's Office of Media and Entertainment (MOME)</t>
+  </si>
+  <si>
+    <t>Mayor's Office of Criminal Justice (MOCJ)</t>
+  </si>
+  <si>
+    <t>Economic Development Corporation (EDC)</t>
+  </si>
+  <si>
+    <t>Department of Information Technology and Telecommunications (DOITT)</t>
+  </si>
+  <si>
+    <t>Department of Buildings (DOB)</t>
+  </si>
+  <si>
+    <t>Department of Consumer and Worker Protection (DCWP)</t>
+  </si>
+  <si>
+    <t>City University of New York (CUNY)</t>
+  </si>
+  <si>
+    <t>Mayor's Office of Citywide Event Coordination and Management (CECM)</t>
+  </si>
+  <si>
+    <t>CUNY</t>
+  </si>
+  <si>
+    <t>CECM</t>
+  </si>
+  <si>
+    <t>Community Board (for SSO)</t>
+  </si>
+  <si>
+    <t>SI99:New Analysis Question:communityBoardID</t>
+  </si>
+  <si>
+    <t>BX1:New Analysis Question:communityBoardID</t>
+  </si>
+  <si>
+    <t>Your FY26 Community District Overview</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -745,9 +989,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -766,9 +1009,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -806,7 +1049,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -912,7 +1155,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1054,7 +1297,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1062,17 +1305,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F02FFFD0-C5F9-B645-9DCF-F351EF9D5B6C}">
-  <dimension ref="A1:B142"/>
+  <dimension ref="A1:B146"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="85.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -1080,7 +1323,7 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -1175,742 +1418,736 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B22" t="s">
-        <v>19</v>
+        <v>210</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" t="s">
-        <v>104</v>
+        <v>300</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" t="s">
-        <v>105</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" t="s">
-        <v>106</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" t="s">
-        <v>107</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>108</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>25</v>
-      </c>
-      <c r="B28" t="s">
-        <v>109</v>
+        <v>301</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>26</v>
+        <v>302</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>27</v>
+        <v>20</v>
+      </c>
+      <c r="B30" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>28</v>
+        <v>21</v>
+      </c>
+      <c r="B31" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>22</v>
+      </c>
+      <c r="B32" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>23</v>
+      </c>
+      <c r="B33" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>31</v>
+        <v>24</v>
+      </c>
+      <c r="B34" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B35" t="s">
-        <v>32</v>
+        <v>107</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>31</v>
+        <v>303</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>37</v>
-      </c>
-      <c r="B40" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>39</v>
-      </c>
-      <c r="B41" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>41</v>
-      </c>
-      <c r="B42" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>43</v>
-      </c>
-      <c r="B43" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="B44" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="B45" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>49</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
+      </c>
+      <c r="B46" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>51</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
+      </c>
+      <c r="B47" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>53</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>52</v>
+        <v>43</v>
+      </c>
+      <c r="B48" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>34</v>
+        <v>45</v>
+      </c>
+      <c r="B49" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>34</v>
+        <v>47</v>
+      </c>
+      <c r="B50" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>35</v>
+        <v>49</v>
+      </c>
+      <c r="B51" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>31</v>
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>54</v>
-      </c>
-      <c r="B53" t="s">
-        <v>128</v>
+        <v>32</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>55</v>
-      </c>
-      <c r="B54" t="s">
-        <v>143</v>
+        <v>32</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>56</v>
-      </c>
-      <c r="B55" t="s">
-        <v>152</v>
+        <v>33</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>57</v>
-      </c>
-      <c r="B56" t="s">
-        <v>110</v>
+        <v>31</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B57" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B58" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B59" t="s">
-        <v>113</v>
+        <v>150</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>34</v>
+        <v>55</v>
+      </c>
+      <c r="B60" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>34</v>
+        <v>56</v>
+      </c>
+      <c r="B61" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>35</v>
+        <v>57</v>
+      </c>
+      <c r="B62" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>31</v>
+        <v>58</v>
+      </c>
+      <c r="B63" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>61</v>
-      </c>
-      <c r="B64" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>62</v>
-      </c>
-      <c r="B65" t="s">
-        <v>144</v>
+        <v>32</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>63</v>
-      </c>
-      <c r="B66" t="s">
-        <v>135</v>
+        <v>33</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>64</v>
-      </c>
-      <c r="B67" t="s">
-        <v>114</v>
+        <v>31</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B68" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>34</v>
+        <v>60</v>
+      </c>
+      <c r="B69" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>34</v>
+        <v>61</v>
+      </c>
+      <c r="B70" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>35</v>
+        <v>62</v>
+      </c>
+      <c r="B71" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>31</v>
+        <v>63</v>
+      </c>
+      <c r="B72" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>66</v>
-      </c>
-      <c r="B73" t="s">
-        <v>129</v>
+        <v>32</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>67</v>
-      </c>
-      <c r="B74" t="s">
-        <v>145</v>
+        <v>32</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>68</v>
-      </c>
-      <c r="B75" t="s">
-        <v>132</v>
+        <v>33</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>69</v>
-      </c>
-      <c r="B76" t="s">
-        <v>116</v>
+        <v>31</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B77" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>34</v>
+        <v>65</v>
+      </c>
+      <c r="B78" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>34</v>
+        <v>66</v>
+      </c>
+      <c r="B79" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>35</v>
+        <v>67</v>
+      </c>
+      <c r="B80" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>31</v>
+        <v>68</v>
+      </c>
+      <c r="B81" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>71</v>
-      </c>
-      <c r="B82" t="s">
-        <v>136</v>
+        <v>32</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>72</v>
-      </c>
-      <c r="B83" t="s">
-        <v>146</v>
+        <v>32</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>73</v>
-      </c>
-      <c r="B84" t="s">
-        <v>137</v>
+        <v>33</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>74</v>
-      </c>
-      <c r="B85" t="s">
-        <v>138</v>
+        <v>31</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B86" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>34</v>
+        <v>70</v>
+      </c>
+      <c r="B87" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>34</v>
+        <v>71</v>
+      </c>
+      <c r="B88" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>35</v>
+        <v>72</v>
+      </c>
+      <c r="B89" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>31</v>
+        <v>73</v>
+      </c>
+      <c r="B90" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>76</v>
-      </c>
-      <c r="B91" t="s">
-        <v>139</v>
+        <v>32</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>77</v>
-      </c>
-      <c r="B92" t="s">
-        <v>147</v>
+        <v>32</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>78</v>
-      </c>
-      <c r="B93" t="s">
-        <v>142</v>
+        <v>33</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>79</v>
-      </c>
-      <c r="B94" t="s">
-        <v>119</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B95" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B96" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>34</v>
+        <v>76</v>
+      </c>
+      <c r="B97" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>34</v>
+        <v>77</v>
+      </c>
+      <c r="B98" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>35</v>
+        <v>78</v>
+      </c>
+      <c r="B99" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>31</v>
+        <v>79</v>
+      </c>
+      <c r="B100" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>82</v>
-      </c>
-      <c r="B101" t="s">
-        <v>130</v>
+        <v>32</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>83</v>
-      </c>
-      <c r="B102" t="s">
-        <v>148</v>
+        <v>32</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>84</v>
-      </c>
-      <c r="B103" t="s">
-        <v>133</v>
+        <v>33</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>85</v>
-      </c>
-      <c r="B104" t="s">
-        <v>122</v>
+        <v>31</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B105" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>34</v>
+        <v>81</v>
+      </c>
+      <c r="B106" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>34</v>
+        <v>82</v>
+      </c>
+      <c r="B107" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>35</v>
+        <v>83</v>
+      </c>
+      <c r="B108" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>31</v>
+        <v>84</v>
+      </c>
+      <c r="B109" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>87</v>
-      </c>
-      <c r="B110" t="s">
-        <v>140</v>
+        <v>32</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>88</v>
-      </c>
-      <c r="B111" t="s">
-        <v>149</v>
+        <v>32</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>89</v>
-      </c>
-      <c r="B112" t="s">
-        <v>141</v>
+        <v>33</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>90</v>
-      </c>
-      <c r="B113" t="s">
-        <v>124</v>
+        <v>31</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B114" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="B115" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B116" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>34</v>
+        <v>88</v>
+      </c>
+      <c r="B117" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>34</v>
+        <v>89</v>
+      </c>
+      <c r="B118" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>35</v>
+        <v>90</v>
+      </c>
+      <c r="B119" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>31</v>
+        <v>91</v>
+      </c>
+      <c r="B120" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>94</v>
-      </c>
-      <c r="B121" t="s">
-        <v>153</v>
+        <v>32</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>31</v>
+        <v>92</v>
+      </c>
+      <c r="B125" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>95</v>
-      </c>
-      <c r="B126" t="s">
-        <v>131</v>
+        <v>32</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>31</v>
+        <v>93</v>
+      </c>
+      <c r="B130" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>96</v>
-      </c>
-      <c r="B131" t="s">
-        <v>96</v>
+        <v>32</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>97</v>
+        <v>32</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
-        <v>98</v>
+        <v>33</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.2">
@@ -1920,41 +2157,64 @@
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>99</v>
+        <v>94</v>
+      </c>
+      <c r="B135" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>31</v>
+        <v>96</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>101</v>
+        <v>31</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>31</v>
+        <v>98</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A143" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A145" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A146" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1965,7 +2225,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6F5E8B0-77B9-4E4F-8066-17FC89ECA64A}">
-  <dimension ref="A1:B67"/>
+  <dimension ref="A1:B72"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="130" bestFit="1" customWidth="1"/>
@@ -1973,17 +2233,17 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -1991,7 +2251,7 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -2086,305 +2346,655 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>19</v>
-      </c>
-      <c r="B23" t="s">
-        <v>19</v>
+        <v>210</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>154</v>
+        <v>19</v>
       </c>
       <c r="B24" t="s">
-        <v>154</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B25" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B26" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B27" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B28" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B29" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B30" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>167</v>
+        <v>164</v>
+      </c>
+      <c r="B31" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>170</v>
-      </c>
-      <c r="B33" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B34" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>173</v>
+        <v>170</v>
+      </c>
+      <c r="B35" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>175</v>
-      </c>
-      <c r="B36" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B37" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B38" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>181</v>
+        <v>211</v>
       </c>
       <c r="B39" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>183</v>
+        <v>212</v>
       </c>
       <c r="B40" t="s">
-        <v>182</v>
+        <v>224</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>185</v>
-      </c>
-      <c r="B41" t="s">
-        <v>184</v>
+        <v>213</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>187</v>
-      </c>
-      <c r="B42" t="s">
-        <v>186</v>
+        <v>214</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>188</v>
+        <v>215</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>190</v>
-      </c>
-      <c r="B44" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="B45" t="s">
-        <v>191</v>
+        <v>177</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="B46" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="B47" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="B48" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="B49" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="B50" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="B51" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>205</v>
+        <v>192</v>
+      </c>
+      <c r="B52" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>206</v>
+        <v>216</v>
+      </c>
+      <c r="B53" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>207</v>
+        <v>217</v>
+      </c>
+      <c r="B54" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>215</v>
+        <v>200</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>220</v>
-      </c>
-      <c r="B67" t="s">
-        <v>220</v>
+        <v>205</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>208</v>
+      </c>
+      <c r="B70" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>219</v>
+      </c>
+      <c r="B72" t="s">
+        <v>222</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4799C399-2879-F546-A0BE-828EB8EDC1C7}">
+  <dimension ref="A1:B39"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="62.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B1" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>261</v>
+      </c>
+      <c r="B2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B4" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>264</v>
+      </c>
+      <c r="B5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>265</v>
+      </c>
+      <c r="B6" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>266</v>
+      </c>
+      <c r="B7" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>267</v>
+      </c>
+      <c r="B8" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>268</v>
+      </c>
+      <c r="B9" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>269</v>
+      </c>
+      <c r="B10" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>270</v>
+      </c>
+      <c r="B11" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>271</v>
+      </c>
+      <c r="B12" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>272</v>
+      </c>
+      <c r="B13" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>273</v>
+      </c>
+      <c r="B14" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>274</v>
+      </c>
+      <c r="B15" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>275</v>
+      </c>
+      <c r="B16" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>276</v>
+      </c>
+      <c r="B17" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>277</v>
+      </c>
+      <c r="B18" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>278</v>
+      </c>
+      <c r="B19" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>279</v>
+      </c>
+      <c r="B20" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>244</v>
+      </c>
+      <c r="B21" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>280</v>
+      </c>
+      <c r="B22" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>281</v>
+      </c>
+      <c r="B23" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>282</v>
+      </c>
+      <c r="B24" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>283</v>
+      </c>
+      <c r="B25" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>284</v>
+      </c>
+      <c r="B26" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>285</v>
+      </c>
+      <c r="B27" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>286</v>
+      </c>
+      <c r="B28" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>287</v>
+      </c>
+      <c r="B29" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>288</v>
+      </c>
+      <c r="B30" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>289</v>
+      </c>
+      <c r="B31" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>290</v>
+      </c>
+      <c r="B32" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>291</v>
+      </c>
+      <c r="B33" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>292</v>
+      </c>
+      <c r="B34" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>293</v>
+      </c>
+      <c r="B35" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>294</v>
+      </c>
+      <c r="B36" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>295</v>
+      </c>
+      <c r="B37" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>296</v>
+      </c>
+      <c r="B38" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>297</v>
+      </c>
+      <c r="B39" t="s">
+        <v>299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added communityDistrictOverview back, which was mistakenly removed
</commit_message>
<xml_diff>
--- a/public/csvdata/variablenamelookups.xlsx
+++ b/public/csvdata/variablenamelookups.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidhochbaum/ae-cd-needs-statements-generator/public/csvdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D6ECA8-101D-9B4A-99B0-3BB1AF96C8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD37F5E3-E3AE-9E4B-9CCA-3CE667510D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49160" yWindow="-4300" windowWidth="26440" windowHeight="15440" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
+    <workbookView xWindow="34600" yWindow="-11200" windowWidth="26440" windowHeight="15440" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Statements" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="305">
   <si>
     <t>Response ID</t>
   </si>
@@ -954,6 +954,9 @@
   </si>
   <si>
     <t>Your FY26 Community District Overview</t>
+  </si>
+  <si>
+    <t>communityDistrictOverview</t>
   </si>
 </sst>
 </file>
@@ -1526,6 +1529,9 @@
       <c r="A39" t="s">
         <v>303</v>
       </c>
+      <c r="B39" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">

</xml_diff>

<commit_message>
Fixes for multi-line responses
</commit_message>
<xml_diff>
--- a/public/csvdata/variablenamelookups.xlsx
+++ b/public/csvdata/variablenamelookups.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidhochbaum/ae-cd-needs-statements-generator/public/csvdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD37F5E3-E3AE-9E4B-9CCA-3CE667510D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F1DB24-2D80-4044-8633-DA1512220D0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34600" yWindow="-11200" windowWidth="26440" windowHeight="15440" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
+    <workbookView xWindow="56460" yWindow="-11200" windowWidth="26240" windowHeight="32260" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Statements" sheetId="1" r:id="rId1"/>
     <sheet name="brs" sheetId="2" r:id="rId2"/>
     <sheet name="Agency Acronyms" sheetId="3" r:id="rId3"/>
+    <sheet name="boro&amp;board" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">brs!$A$1:$B$72</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Statements!$A$1:$B$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Statements!$A$1:$E$147</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="388">
   <si>
     <t>Response ID</t>
   </si>
@@ -957,19 +958,282 @@
   </si>
   <si>
     <t>communityDistrictOverview</t>
+  </si>
+  <si>
+    <t>Export Header</t>
+  </si>
+  <si>
+    <t>Variable Name</t>
+  </si>
+  <si>
+    <t>Question #</t>
+  </si>
+  <si>
+    <t>question(102), option("10830-other")</t>
+  </si>
+  <si>
+    <t>question(100), option("10805-other")</t>
+  </si>
+  <si>
+    <t>question(98), option("10780-other")</t>
+  </si>
+  <si>
+    <t>question(106), option("10844-other")</t>
+  </si>
+  <si>
+    <t>question(110), option("10860-other")</t>
+  </si>
+  <si>
+    <t>question(113), option("10872-other")</t>
+  </si>
+  <si>
+    <t>question(116), option("10887-other")</t>
+  </si>
+  <si>
+    <t>question(119), option("10901-other")</t>
+  </si>
+  <si>
+    <t>question(122), option("10916-other")</t>
+  </si>
+  <si>
+    <t>question(125), option("10931-other")</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>For LUA</t>
+  </si>
+  <si>
+    <t>responseID</t>
+  </si>
+  <si>
+    <t>SI99</t>
+  </si>
+  <si>
+    <t>BX1</t>
+  </si>
+  <si>
+    <t>BX2</t>
+  </si>
+  <si>
+    <t>BX3</t>
+  </si>
+  <si>
+    <t>BX4</t>
+  </si>
+  <si>
+    <t>BX5</t>
+  </si>
+  <si>
+    <t>BX6</t>
+  </si>
+  <si>
+    <t>BX7</t>
+  </si>
+  <si>
+    <t>BX8</t>
+  </si>
+  <si>
+    <t>BX9</t>
+  </si>
+  <si>
+    <t>BX10</t>
+  </si>
+  <si>
+    <t>BX11</t>
+  </si>
+  <si>
+    <t>BX12</t>
+  </si>
+  <si>
+    <t>BK1</t>
+  </si>
+  <si>
+    <t>BK2</t>
+  </si>
+  <si>
+    <t>BK3</t>
+  </si>
+  <si>
+    <t>BK4</t>
+  </si>
+  <si>
+    <t>BK5</t>
+  </si>
+  <si>
+    <t>BK6</t>
+  </si>
+  <si>
+    <t>BK7</t>
+  </si>
+  <si>
+    <t>BK8</t>
+  </si>
+  <si>
+    <t>BK9</t>
+  </si>
+  <si>
+    <t>BK10</t>
+  </si>
+  <si>
+    <t>BK11</t>
+  </si>
+  <si>
+    <t>BK12</t>
+  </si>
+  <si>
+    <t>BK13</t>
+  </si>
+  <si>
+    <t>BK14</t>
+  </si>
+  <si>
+    <t>BK15</t>
+  </si>
+  <si>
+    <t>BK16</t>
+  </si>
+  <si>
+    <t>BK17</t>
+  </si>
+  <si>
+    <t>BK18</t>
+  </si>
+  <si>
+    <t>MN1</t>
+  </si>
+  <si>
+    <t>MN2</t>
+  </si>
+  <si>
+    <t>MN3</t>
+  </si>
+  <si>
+    <t>MN4</t>
+  </si>
+  <si>
+    <t>MN5</t>
+  </si>
+  <si>
+    <t>MN6</t>
+  </si>
+  <si>
+    <t>MN7</t>
+  </si>
+  <si>
+    <t>MN8</t>
+  </si>
+  <si>
+    <t>MN9</t>
+  </si>
+  <si>
+    <t>MN10</t>
+  </si>
+  <si>
+    <t>MN11</t>
+  </si>
+  <si>
+    <t>MN12</t>
+  </si>
+  <si>
+    <t>QN1</t>
+  </si>
+  <si>
+    <t>QN2</t>
+  </si>
+  <si>
+    <t>QN3</t>
+  </si>
+  <si>
+    <t>QN4</t>
+  </si>
+  <si>
+    <t>QN5</t>
+  </si>
+  <si>
+    <t>QN6</t>
+  </si>
+  <si>
+    <t>QN7</t>
+  </si>
+  <si>
+    <t>QN8</t>
+  </si>
+  <si>
+    <t>QN9</t>
+  </si>
+  <si>
+    <t>QN10</t>
+  </si>
+  <si>
+    <t>QN11</t>
+  </si>
+  <si>
+    <t>QN12</t>
+  </si>
+  <si>
+    <t>QN13</t>
+  </si>
+  <si>
+    <t>QN14</t>
+  </si>
+  <si>
+    <t>SI1</t>
+  </si>
+  <si>
+    <t>SI2</t>
+  </si>
+  <si>
+    <t>SI3</t>
+  </si>
+  <si>
+    <t>Board</t>
+  </si>
+  <si>
+    <t>Staten Island</t>
+  </si>
+  <si>
+    <t>Queens</t>
+  </si>
+  <si>
+    <t>Manhattan</t>
+  </si>
+  <si>
+    <t>Brooklyn</t>
+  </si>
+  <si>
+    <t>Bronx</t>
+  </si>
+  <si>
+    <t>Boro</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -992,8 +1256,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1308,924 +1574,1815 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F02FFFD0-C5F9-B645-9DCF-F351EF9D5B6C}">
-  <dimension ref="A1:B146"/>
+  <dimension ref="A1:E147"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="85.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B1" t="s">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B2" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>0</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C4" t="s">
+        <v>320</v>
+      </c>
+      <c r="D4" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="E4" t="str">
+        <f>"x["""&amp;D4&amp;"""] = v["""&amp;C4&amp;"""];"</f>
+        <v>x["responseId"] = v["responseID"];</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
         <v>19</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C28">
+        <v>283</v>
+      </c>
+      <c r="D28" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+      <c r="E28" t="str">
+        <f>"x["""&amp;D28&amp;"""] = v[""[question("&amp;C28&amp;")]""];"</f>
+        <v>x["communityBoardID"] = v["[question(283)]"];</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
         <v>20</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C31">
+        <v>89</v>
+      </c>
+      <c r="D31" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+      <c r="E31" t="str">
+        <f>"x["""&amp;D31&amp;"""] = v[""[question("&amp;C31&amp;")]""];"</f>
+        <v>x["communityBoardChair"] = v["[question(89)]"];</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
         <v>21</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C32">
+        <v>90</v>
+      </c>
+      <c r="D32" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+      <c r="E32" t="str">
+        <f>"x["""&amp;D32&amp;"""] = v[""[question("&amp;C32&amp;")]""];"</f>
+        <v>x["districtManager"] = v["[question(90)]"];</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
         <v>22</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C33">
+        <v>91</v>
+      </c>
+      <c r="D33" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+      <c r="E33" t="str">
+        <f>"x["""&amp;D33&amp;"""] = v[""[question("&amp;C33&amp;")]""];"</f>
+        <v>x["communityBoardOfficeAddress"] = v["[question(91)]"];</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
         <v>23</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C34">
+        <v>92</v>
+      </c>
+      <c r="D34" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="E34" t="str">
+        <f>"x["""&amp;D34&amp;"""] = v[""[question("&amp;C34&amp;")]""];"</f>
+        <v>x["communityBoardOfficePhoneNumber"] = v["[question(92)]"];</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
         <v>24</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C35">
+        <v>93</v>
+      </c>
+      <c r="D35" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="E35" t="str">
+        <f>"x["""&amp;D35&amp;"""] = v[""[question("&amp;C35&amp;")]""];"</f>
+        <v>x["communityBoardOfficeEmailAddress"] = v["[question(93)]"];</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
         <v>25</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C36">
+        <v>94</v>
+      </c>
+      <c r="D36" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
+      <c r="E36" t="str">
+        <f>"x["""&amp;D36&amp;"""] = v[""[question("&amp;C36&amp;")]""];"</f>
+        <v>x["communityBoardWebsiteUrl"] = v["[question(94)]"];</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
         <v>303</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C40">
+        <v>96</v>
+      </c>
+      <c r="D40" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="E40" t="str">
+        <f>"x["""&amp;D40&amp;"""] = v[""[question("&amp;C40&amp;")]""];"</f>
+        <v>x["communityDistrictOverview"] = v["[question(96)]"];</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
         <v>35</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C45">
+        <v>98</v>
+      </c>
+      <c r="D45" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+      <c r="E45" t="str">
+        <f>"x["""&amp;D45&amp;"""] = v[""[question("&amp;C45&amp;")]""];"</f>
+        <v>x["top3Issues1"] = v["[question(98)]"];</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
         <v>37</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C46" t="s">
+        <v>310</v>
+      </c>
+      <c r="D46" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+      <c r="E46" t="str">
+        <f>"x["""&amp;D46&amp;"""] = v['["&amp;C46&amp;"]'];"</f>
+        <v>x["top3Issues1Other"] = v['[question(98), option("10780-other")]'];</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
         <v>39</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C47">
+        <v>99</v>
+      </c>
+      <c r="D47" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+      <c r="E47" t="str">
+        <f>"x["""&amp;D47&amp;"""] = v[""[question("&amp;C47&amp;")]""];"</f>
+        <v>x["top3Issues1Explanation"] = v["[question(99)]"];</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
         <v>41</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C48">
+        <v>100</v>
+      </c>
+      <c r="D48" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+      <c r="E48" t="str">
+        <f>"x["""&amp;D48&amp;"""] = v[""[question("&amp;C48&amp;")]""];"</f>
+        <v>x["top3Issues2"] = v["[question(100)]"];</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
         <v>43</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C49" t="s">
+        <v>309</v>
+      </c>
+      <c r="D49" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+      <c r="E49" t="str">
+        <f>"x["""&amp;D49&amp;"""] = v['["&amp;C49&amp;"]'];"</f>
+        <v>x["top3Issues2Other"] = v['[question(100), option("10805-other")]'];</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
         <v>45</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C50">
+        <v>101</v>
+      </c>
+      <c r="D50" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
+      <c r="E50" t="str">
+        <f>"x["""&amp;D50&amp;"""] = v[""[question("&amp;C50&amp;")]""];"</f>
+        <v>x["top3Issues2Explanation"] = v["[question(101)]"];</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
         <v>47</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C51">
+        <v>102</v>
+      </c>
+      <c r="D51" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+      <c r="E51" t="str">
+        <f>"x["""&amp;D51&amp;"""] = v[""[question("&amp;C51&amp;")]""];"</f>
+        <v>x["top3Issues3"] = v["[question(102)]"];</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
         <v>49</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C52" t="s">
+        <v>308</v>
+      </c>
+      <c r="D52" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+      <c r="E52" t="str">
+        <f>"x["""&amp;D52&amp;"""] = v['["&amp;C52&amp;"]'];"</f>
+        <v>x["top3Issues3Other"] = v['[question(102), option("10830-other")]'];</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
         <v>51</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C53">
+        <v>103</v>
+      </c>
+      <c r="D53" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+      <c r="E53" t="str">
+        <f>"x["""&amp;D53&amp;"""] = v[""[question("&amp;C53&amp;")]""];"</f>
+        <v>x["top3Issues3Explanation"] = v["[question(103)]"];</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
         <v>52</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C58">
+        <v>106</v>
+      </c>
+      <c r="D58" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
+      <c r="E58" t="str">
+        <f>"x["""&amp;D58&amp;"""] = v[""[question("&amp;C58&amp;")]""];"</f>
+        <v>x["mostImportantIssueHealthcareAndHumanServices"] = v["[question(106)]"];</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
         <v>53</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C59" t="s">
+        <v>311</v>
+      </c>
+      <c r="D59" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
+      <c r="E59" t="str">
+        <f>"x["""&amp;D59&amp;"""] = v['["&amp;C59&amp;"]'];"</f>
+        <v>x["mostImportantIssueHealthcareAndHumanServicesOther"] = v['[question(106), option("10844-other")]'];</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
         <v>54</v>
       </c>
-      <c r="B59" t="s">
+      <c r="C60">
+        <v>107</v>
+      </c>
+      <c r="D60" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
+      <c r="E60" t="str">
+        <f>"x["""&amp;D60&amp;"""] = v[""[question("&amp;C60&amp;")]""];"</f>
+        <v>x["pleaseExplainYourSelectionForMostImportantIssueInHealthcareAndHumanServices"] = v["[question(107)]"];</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
         <v>55</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C61">
+        <v>144</v>
+      </c>
+      <c r="D61" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
+      <c r="E61" t="str">
+        <f>"x["""&amp;D61&amp;"""] = v[""[question("&amp;C61&amp;")]""];"</f>
+        <v>x["needsForHealthCareAndFacilities"] = v["[question(144)]"];</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
         <v>56</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C62">
+        <v>146</v>
+      </c>
+      <c r="D62" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
+      <c r="E62" t="str">
+        <f>"x["""&amp;D62&amp;"""] = v[""[question("&amp;C62&amp;")]""];"</f>
+        <v>x["needsForOlderNewYorkers"] = v["[question(146)]"];</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
         <v>57</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C63">
+        <v>147</v>
+      </c>
+      <c r="D63" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
+      <c r="E63" t="str">
+        <f>"x["""&amp;D63&amp;"""] = v[""[question("&amp;C63&amp;")]""];"</f>
+        <v>x["needsForHomeless"] = v["[question(147)]"];</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
         <v>58</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C64">
+        <v>148</v>
+      </c>
+      <c r="D64" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
+      <c r="E64" t="str">
+        <f>"x["""&amp;D64&amp;"""] = v[""[question("&amp;C64&amp;")]""];"</f>
+        <v>x["needsForLowIncomeNewYorkers"] = v["[question(148)]"];</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
         <v>59</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C69">
+        <v>110</v>
+      </c>
+      <c r="D69" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
+      <c r="E69" t="str">
+        <f>"x["""&amp;D69&amp;"""] = v[""[question("&amp;C69&amp;")]""];"</f>
+        <v>x["mostImportantIssueYouthEducationAndChildWelfare"] = v["[question(110)]"];</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
         <v>60</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C70" t="s">
+        <v>312</v>
+      </c>
+      <c r="D70" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
+      <c r="E70" t="str">
+        <f>"x["""&amp;D70&amp;"""] = v['["&amp;C70&amp;"]'];"</f>
+        <v>x["mostImportantIssueYouthEducationAndChildWelfareOther"] = v['[question(110), option("10860-other")]'];</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
         <v>61</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C71">
+        <v>111</v>
+      </c>
+      <c r="D71" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
+      <c r="E71" t="str">
+        <f>"x["""&amp;D71&amp;"""] = v[""[question("&amp;C71&amp;")]""];"</f>
+        <v>x["pleaseExplainYourSelectionForMostImportantIssueInYouthEducationAndChildWelfareIssues"] = v["[question(111)]"];</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
         <v>62</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C72">
+        <v>150</v>
+      </c>
+      <c r="D72" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
+      <c r="E72" t="str">
+        <f>"x["""&amp;D72&amp;"""] = v[""[question("&amp;C72&amp;")]""];"</f>
+        <v>x["needsForYouthEducation"] = v["[question(150)]"];</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
         <v>63</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C73">
+        <v>152</v>
+      </c>
+      <c r="D73" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
+      <c r="E73" t="str">
+        <f>"x["""&amp;D73&amp;"""] = v[""[question("&amp;C73&amp;")]""];"</f>
+        <v>x["needsForYouthAndChildWelfare"] = v["[question(152)]"];</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
         <v>64</v>
       </c>
-      <c r="B77" t="s">
+      <c r="C78">
+        <v>113</v>
+      </c>
+      <c r="D78" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
+      <c r="E78" t="str">
+        <f>"x["""&amp;D78&amp;"""] = v[""[question("&amp;C78&amp;")]""];"</f>
+        <v>x["mostImportantIssuePublicSafetyAndEmergencyServices"] = v["[question(113)]"];</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
         <v>65</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C79" t="s">
+        <v>313</v>
+      </c>
+      <c r="D79" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
+      <c r="E79" t="str">
+        <f>"x["""&amp;D79&amp;"""] = v['["&amp;C79&amp;"]'];"</f>
+        <v>x["mostImportantIssuePublicSafetyAndEmergencyServicesOther"] = v['[question(113), option("10872-other")]'];</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
         <v>66</v>
       </c>
-      <c r="B79" t="s">
+      <c r="C80">
+        <v>114</v>
+      </c>
+      <c r="D80" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
+      <c r="E80" t="str">
+        <f>"x["""&amp;D80&amp;"""] = v[""[question("&amp;C80&amp;")]""];"</f>
+        <v>x["pleaseExplainYourSelectionForMostImportantPublicSafetyAndEmergencyServicesIssue"] = v["[question(114)]"];</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
         <v>67</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C81">
+        <v>154</v>
+      </c>
+      <c r="D81" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
+      <c r="E81" t="str">
+        <f>"x["""&amp;D81&amp;"""] = v[""[question("&amp;C81&amp;")]""];"</f>
+        <v>x["needsForPublicSafety"] = v["[question(154)]"];</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
         <v>68</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C82">
+        <v>155</v>
+      </c>
+      <c r="D82" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
+      <c r="E82" t="str">
+        <f>"x["""&amp;D82&amp;"""] = v[""[question("&amp;C82&amp;")]""];"</f>
+        <v>x["needsForEmergencyServices"] = v["[question(155)]"];</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
         <v>69</v>
       </c>
-      <c r="B86" t="s">
+      <c r="C87">
+        <v>116</v>
+      </c>
+      <c r="D87" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
+      <c r="E87" t="str">
+        <f>"x["""&amp;D87&amp;"""] = v[""[question("&amp;C87&amp;")]""];"</f>
+        <v>x["mostImportantIssueCoreInfrastructureCityServicesAndResiliency"] = v["[question(116)]"];</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
         <v>70</v>
       </c>
-      <c r="B87" t="s">
+      <c r="C88" t="s">
+        <v>314</v>
+      </c>
+      <c r="D88" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
+      <c r="E88" t="str">
+        <f>"x["""&amp;D88&amp;"""] = v['["&amp;C88&amp;"]'];"</f>
+        <v>x["mostImportantIssueCoreInfrastructureCityServicesAndResiliencyOther"] = v['[question(116), option("10887-other")]'];</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
         <v>71</v>
       </c>
-      <c r="B88" t="s">
+      <c r="C89">
+        <v>117</v>
+      </c>
+      <c r="D89" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
+      <c r="E89" t="str">
+        <f>"x["""&amp;D89&amp;"""] = v[""[question("&amp;C89&amp;")]""];"</f>
+        <v>x["pleaseExplainYourSelectionForMostImportantCoreInfrastructureCityServicesAndResiliencyIssue"] = v["[question(117)]"];</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
         <v>72</v>
       </c>
-      <c r="B89" t="s">
+      <c r="C90">
+        <v>157</v>
+      </c>
+      <c r="D90" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
+      <c r="E90" t="str">
+        <f>"x["""&amp;D90&amp;"""] = v[""[question("&amp;C90&amp;")]""];"</f>
+        <v>x["needsForWaterSewersAndEnvironmentalProtection"] = v["[question(157)]"];</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
         <v>73</v>
       </c>
-      <c r="B90" t="s">
+      <c r="C91">
+        <v>158</v>
+      </c>
+      <c r="D91" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
+      <c r="E91" t="str">
+        <f>"x["""&amp;D91&amp;"""] = v[""[question("&amp;C91&amp;")]""];"</f>
+        <v>x["needsForSanitationServices"] = v["[question(158)]"];</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="s">
         <v>74</v>
       </c>
-      <c r="B95" t="s">
+      <c r="C96">
+        <v>119</v>
+      </c>
+      <c r="D96" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
+      <c r="E96" t="str">
+        <f>"x["""&amp;D96&amp;"""] = v[""[question("&amp;C96&amp;")]""];"</f>
+        <v>x["mostImportantIssueHousingEconomicDevelopmentAndLandUse"] = v["[question(119)]"];</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
         <v>75</v>
       </c>
-      <c r="B96" t="s">
+      <c r="C97" t="s">
+        <v>315</v>
+      </c>
+      <c r="D97" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
+      <c r="E97" t="str">
+        <f>"x["""&amp;D97&amp;"""] = v['["&amp;C97&amp;"]'];"</f>
+        <v>x["mostImportantIssueHousingEconomicDevelopmentAndLandUseOther"] = v['[question(119), option("10901-other")]'];</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
         <v>76</v>
       </c>
-      <c r="B97" t="s">
+      <c r="C98">
+        <v>120</v>
+      </c>
+      <c r="D98" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
+      <c r="E98" t="str">
+        <f>"x["""&amp;D98&amp;"""] = v[""[question("&amp;C98&amp;")]""];"</f>
+        <v>x["pleaseExplainYourSelectionForMostImportantHousingEconomicDevelopmentAndHousingIssue"] = v["[question(120)]"];</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="s">
         <v>77</v>
       </c>
-      <c r="B98" t="s">
+      <c r="C99">
+        <v>161</v>
+      </c>
+      <c r="D99" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
+      <c r="E99" t="str">
+        <f>"x["""&amp;D99&amp;"""] = v[""[question("&amp;C99&amp;")]""];"</f>
+        <v>x["needsForLandUse"] = v["[question(161)]"];</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="s">
         <v>78</v>
       </c>
-      <c r="B99" t="s">
+      <c r="C100">
+        <v>162</v>
+      </c>
+      <c r="D100" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
+      <c r="E100" t="str">
+        <f>"x["""&amp;D100&amp;"""] = v[""[question("&amp;C100&amp;")]""];"</f>
+        <v>x["needsForHousing"] = v["[question(162)]"];</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" t="s">
         <v>79</v>
       </c>
-      <c r="B100" t="s">
+      <c r="C101">
+        <v>163</v>
+      </c>
+      <c r="D101" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
+      <c r="E101" t="str">
+        <f>"x["""&amp;D101&amp;"""] = v[""[question("&amp;C101&amp;")]""];"</f>
+        <v>x["needsForEconomicDevelopment"] = v["[question(163)]"];</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A104" t="s">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106" t="s">
         <v>80</v>
       </c>
-      <c r="B105" t="s">
+      <c r="C106">
+        <v>122</v>
+      </c>
+      <c r="D106" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
+      <c r="E106" t="str">
+        <f>"x["""&amp;D106&amp;"""] = v[""[question("&amp;C106&amp;")]""];"</f>
+        <v>x["mostImportantIssueTransportationAndMobility"] = v["[question(122)]"];</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107" t="s">
         <v>81</v>
       </c>
-      <c r="B106" t="s">
+      <c r="C107" t="s">
+        <v>316</v>
+      </c>
+      <c r="D107" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A107" t="s">
+      <c r="E107" t="str">
+        <f>"x["""&amp;D107&amp;"""] = v['["&amp;C107&amp;"]'];"</f>
+        <v>x["mostImportantIssueTransportationAndMobilityOther"] = v['[question(122), option("10916-other")]'];</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108" t="s">
         <v>82</v>
       </c>
-      <c r="B107" t="s">
+      <c r="C108">
+        <v>123</v>
+      </c>
+      <c r="D108" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A108" t="s">
+      <c r="E108" t="str">
+        <f>"x["""&amp;D108&amp;"""] = v[""[question("&amp;C108&amp;")]""];"</f>
+        <v>x["pleaseExplainYourSelectionForMostImportantTransportationAndMobilityIssue"] = v["[question(123)]"];</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109" t="s">
         <v>83</v>
       </c>
-      <c r="B108" t="s">
+      <c r="C109">
+        <v>165</v>
+      </c>
+      <c r="D109" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
+      <c r="E109" t="str">
+        <f>"x["""&amp;D109&amp;"""] = v[""[question("&amp;C109&amp;")]""];"</f>
+        <v>x["needsForTrafficAndTransportationInfrastructure"] = v["[question(165)]"];</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110" t="s">
         <v>84</v>
       </c>
-      <c r="B109" t="s">
+      <c r="C110">
+        <v>167</v>
+      </c>
+      <c r="D110" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A110" t="s">
+      <c r="E110" t="str">
+        <f>"x["""&amp;D110&amp;"""] = v[""[question("&amp;C110&amp;")]""];"</f>
+        <v>x["needsForTransitServices"] = v["[question(167)]"];</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A113" t="s">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A114">
+        <v>113</v>
+      </c>
+      <c r="B114" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115" t="s">
         <v>85</v>
       </c>
-      <c r="B114" t="s">
+      <c r="C115">
+        <v>125</v>
+      </c>
+      <c r="D115" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
+      <c r="E115" t="str">
+        <f>"x["""&amp;D115&amp;"""] = v[""[question("&amp;C115&amp;")]""];"</f>
+        <v>x["mostImportantIssueParksCulturalAndOtherCommunityFacilities"] = v["[question(125)]"];</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116" t="s">
         <v>86</v>
       </c>
-      <c r="B115" t="s">
+      <c r="C116" t="s">
+        <v>317</v>
+      </c>
+      <c r="D116" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A116" t="s">
+      <c r="E116" t="str">
+        <f>"x["""&amp;D116&amp;"""] = v['["&amp;C116&amp;"]'];"</f>
+        <v>x["mostImportantIssueParksCulturalAndOtherCommunityFacilitiesOther"] = v['[question(125), option("10931-other")]'];</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117" t="s">
         <v>87</v>
       </c>
-      <c r="B116" t="s">
+      <c r="C117">
+        <v>126</v>
+      </c>
+      <c r="D117" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A117" t="s">
+      <c r="E117" t="str">
+        <f>"x["""&amp;D117&amp;"""] = v[""[question("&amp;C117&amp;")]""];"</f>
+        <v>x["pleaseExplainYourSelectionForMostImportantParksCulturalAndOtherCommunityFacilitiesIssue"] = v["[question(126)]"];</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118" t="s">
         <v>88</v>
       </c>
-      <c r="B117" t="s">
+      <c r="C118">
+        <v>169</v>
+      </c>
+      <c r="D118" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A118" t="s">
+      <c r="E118" t="str">
+        <f>"x["""&amp;D118&amp;"""] = v[""[question("&amp;C118&amp;")]""];"</f>
+        <v>x["needsForParks"] = v["[question(169)]"];</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119" t="s">
         <v>89</v>
       </c>
-      <c r="B118" t="s">
+      <c r="C119">
+        <v>170</v>
+      </c>
+      <c r="D119" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A119" t="s">
+      <c r="E119" t="str">
+        <f>"x["""&amp;D119&amp;"""] = v[""[question("&amp;C119&amp;")]""];"</f>
+        <v>x["needsForCulturalServices"] = v["[question(170)]"];</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120" t="s">
         <v>90</v>
       </c>
-      <c r="B119" t="s">
+      <c r="C120">
+        <v>171</v>
+      </c>
+      <c r="D120" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A120" t="s">
+      <c r="E120" t="str">
+        <f>"x["""&amp;D120&amp;"""] = v[""[question("&amp;C120&amp;")]""];"</f>
+        <v>x["needsForLibraryServices"] = v["[question(171)]"];</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121" t="s">
         <v>91</v>
       </c>
-      <c r="B120" t="s">
+      <c r="C121">
+        <v>172</v>
+      </c>
+      <c r="D121" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A121" t="s">
+      <c r="E121" t="str">
+        <f>"x["""&amp;D121&amp;"""] = v[""[question("&amp;C121&amp;")]""];"</f>
+        <v>x["needsForCommunityBoards"] = v["[question(172)]"];</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A122">
+        <v>121</v>
+      </c>
+      <c r="B122" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A122" t="s">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A123">
+        <v>122</v>
+      </c>
+      <c r="B123" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A123" t="s">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A124">
+        <v>123</v>
+      </c>
+      <c r="B124" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A124" t="s">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A125">
+        <v>124</v>
+      </c>
+      <c r="B125" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A125" t="s">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A126">
+        <v>125</v>
+      </c>
+      <c r="B126" t="s">
         <v>92</v>
       </c>
-      <c r="B125" t="s">
+      <c r="C126">
+        <v>127</v>
+      </c>
+      <c r="D126" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A126" t="s">
+      <c r="E126" t="str">
+        <f>"x["""&amp;D126&amp;"""] = v[""[question("&amp;C126&amp;")]""];"</f>
+        <v>x["anyNeedsNotDetailedInThePrecedingPolicyArea"] = v["[question(127)]"];</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A127">
+        <v>126</v>
+      </c>
+      <c r="B127" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A127" t="s">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A128" t="s">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A129" t="s">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A130" t="s">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131" t="s">
         <v>93</v>
       </c>
-      <c r="B130" t="s">
+      <c r="C131">
+        <v>128</v>
+      </c>
+      <c r="D131" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A131" t="s">
+      <c r="E131" t="str">
+        <f>"x["""&amp;D131&amp;"""] = v[""[question("&amp;C131&amp;")]""];"</f>
+        <v>x["anyAdditionalCommentsRelatedToYourDistrictsNeedsAndBudgetRequests"] = v["[question(128)]"];</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A132" t="s">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A133" t="s">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A134" t="s">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A135" t="s">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136" t="s">
         <v>94</v>
       </c>
-      <c r="B135" t="s">
+      <c r="C136">
+        <v>77</v>
+      </c>
+      <c r="D136" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A136" t="s">
+      <c r="E136" t="str">
+        <f>"x["""&amp;D136&amp;"""] = v[""[question("&amp;C136&amp;")]""];"</f>
+        <v>x["cb"] = v["[question(77)]"];</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A137" t="s">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A138" t="s">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A139" t="s">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A140" t="s">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A141" t="s">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A142" t="s">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A143">
+        <v>142</v>
+      </c>
+      <c r="B143" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A143" t="s">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A144">
+        <v>143</v>
+      </c>
+      <c r="B144" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A144" t="s">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A145">
+        <v>144</v>
+      </c>
+      <c r="B145" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A145" t="s">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A146">
+        <v>145</v>
+      </c>
+      <c r="B146" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A146" t="s">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A147">
+        <v>146</v>
+      </c>
+      <c r="B147" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E147" xr:uid="{F02FFFD0-C5F9-B645-9DCF-F351EF9D5B6C}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E147">
+    <sortCondition ref="A2:A147"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -3006,4 +4163,1229 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E64C24E-6C75-9B4A-AA22-C3274D2524A0}">
+  <dimension ref="A1:G62"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B1" t="s">
+        <v>387</v>
+      </c>
+      <c r="C1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B2" t="s">
+        <v>382</v>
+      </c>
+      <c r="C2" t="str">
+        <f>RIGHT(A2,LEN(A2)-2)</f>
+        <v>99</v>
+      </c>
+      <c r="E2" t="str">
+        <f>"boros["""&amp;A2&amp;"""] = """&amp;B2&amp;""";"</f>
+        <v>boros["SI99"] = "Staten Island";</v>
+      </c>
+      <c r="G2" t="str">
+        <f>"boards["""&amp;A2&amp;"""] = """&amp;C2&amp;""";"</f>
+        <v>boards["SI99"] = "99";</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C3" t="str">
+        <f t="shared" ref="C3:C61" si="0">RIGHT(A3,LEN(A3)-2)</f>
+        <v>1</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E61" si="1">"boros["""&amp;A3&amp;"""] = """&amp;B3&amp;""";"</f>
+        <v>boros["BX1"] = "Bronx";</v>
+      </c>
+      <c r="G3" t="str">
+        <f t="shared" ref="G3:G61" si="2">"boards["""&amp;A3&amp;"""] = """&amp;C3&amp;""";"</f>
+        <v>boards["BX1"] = "1";</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="B4" t="s">
+        <v>386</v>
+      </c>
+      <c r="C4" t="str">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BX2"] = "Bronx";</v>
+      </c>
+      <c r="G4" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BX2"] = "2";</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B5" t="s">
+        <v>386</v>
+      </c>
+      <c r="C5" t="str">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BX3"] = "Bronx";</v>
+      </c>
+      <c r="G5" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BX3"] = "3";</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="B6" t="s">
+        <v>386</v>
+      </c>
+      <c r="C6" t="str">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BX4"] = "Bronx";</v>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BX4"] = "4";</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B7" t="s">
+        <v>386</v>
+      </c>
+      <c r="C7" t="str">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E7" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BX5"] = "Bronx";</v>
+      </c>
+      <c r="G7" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BX5"] = "5";</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B8" t="s">
+        <v>386</v>
+      </c>
+      <c r="C8" t="str">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="E8" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BX6"] = "Bronx";</v>
+      </c>
+      <c r="G8" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BX6"] = "6";</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B9" t="s">
+        <v>386</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BX7"] = "Bronx";</v>
+      </c>
+      <c r="G9" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BX7"] = "7";</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B10" t="s">
+        <v>386</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BX8"] = "Bronx";</v>
+      </c>
+      <c r="G10" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BX8"] = "8";</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B11" t="s">
+        <v>386</v>
+      </c>
+      <c r="C11" t="str">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="E11" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BX9"] = "Bronx";</v>
+      </c>
+      <c r="G11" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BX9"] = "9";</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="B12" t="s">
+        <v>386</v>
+      </c>
+      <c r="C12" t="str">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="E12" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BX10"] = "Bronx";</v>
+      </c>
+      <c r="G12" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BX10"] = "10";</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="B13" t="s">
+        <v>386</v>
+      </c>
+      <c r="C13" t="str">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="E13" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BX11"] = "Bronx";</v>
+      </c>
+      <c r="G13" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BX11"] = "11";</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B14" t="s">
+        <v>386</v>
+      </c>
+      <c r="C14" t="str">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BX12"] = "Bronx";</v>
+      </c>
+      <c r="G14" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BX12"] = "12";</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="B15" t="s">
+        <v>385</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E15" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK1"] = "Brooklyn";</v>
+      </c>
+      <c r="G15" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK1"] = "1";</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="B16" t="s">
+        <v>385</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E16" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK2"] = "Brooklyn";</v>
+      </c>
+      <c r="G16" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK2"] = "2";</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B17" t="s">
+        <v>385</v>
+      </c>
+      <c r="C17" t="str">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E17" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK3"] = "Brooklyn";</v>
+      </c>
+      <c r="G17" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK3"] = "3";</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B18" t="s">
+        <v>385</v>
+      </c>
+      <c r="C18" t="str">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E18" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK4"] = "Brooklyn";</v>
+      </c>
+      <c r="G18" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK4"] = "4";</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="B19" t="s">
+        <v>385</v>
+      </c>
+      <c r="C19" t="str">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E19" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK5"] = "Brooklyn";</v>
+      </c>
+      <c r="G19" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK5"] = "5";</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B20" t="s">
+        <v>385</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="E20" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK6"] = "Brooklyn";</v>
+      </c>
+      <c r="G20" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK6"] = "6";</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="B21" t="s">
+        <v>385</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK7"] = "Brooklyn";</v>
+      </c>
+      <c r="G21" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK7"] = "7";</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="B22" t="s">
+        <v>385</v>
+      </c>
+      <c r="C22" t="str">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="E22" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK8"] = "Brooklyn";</v>
+      </c>
+      <c r="G22" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK8"] = "8";</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B23" t="s">
+        <v>385</v>
+      </c>
+      <c r="C23" t="str">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="E23" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK9"] = "Brooklyn";</v>
+      </c>
+      <c r="G23" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK9"] = "9";</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="B24" t="s">
+        <v>385</v>
+      </c>
+      <c r="C24" t="str">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="E24" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK10"] = "Brooklyn";</v>
+      </c>
+      <c r="G24" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK10"] = "10";</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="B25" t="s">
+        <v>385</v>
+      </c>
+      <c r="C25" t="str">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="E25" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK11"] = "Brooklyn";</v>
+      </c>
+      <c r="G25" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK11"] = "11";</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B26" t="s">
+        <v>385</v>
+      </c>
+      <c r="C26" t="str">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="E26" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK12"] = "Brooklyn";</v>
+      </c>
+      <c r="G26" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK12"] = "12";</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="B27" t="s">
+        <v>385</v>
+      </c>
+      <c r="C27" t="str">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="E27" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK13"] = "Brooklyn";</v>
+      </c>
+      <c r="G27" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK13"] = "13";</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="B28" t="s">
+        <v>385</v>
+      </c>
+      <c r="C28" t="str">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="E28" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK14"] = "Brooklyn";</v>
+      </c>
+      <c r="G28" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK14"] = "14";</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="B29" t="s">
+        <v>385</v>
+      </c>
+      <c r="C29" t="str">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="E29" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK15"] = "Brooklyn";</v>
+      </c>
+      <c r="G29" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK15"] = "15";</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="B30" t="s">
+        <v>385</v>
+      </c>
+      <c r="C30" t="str">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="E30" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK16"] = "Brooklyn";</v>
+      </c>
+      <c r="G30" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK16"] = "16";</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="B31" t="s">
+        <v>385</v>
+      </c>
+      <c r="C31" t="str">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="E31" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK17"] = "Brooklyn";</v>
+      </c>
+      <c r="G31" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK17"] = "17";</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B32" t="s">
+        <v>385</v>
+      </c>
+      <c r="C32" t="str">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="E32" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["BK18"] = "Brooklyn";</v>
+      </c>
+      <c r="G32" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["BK18"] = "18";</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="B33" t="s">
+        <v>384</v>
+      </c>
+      <c r="C33" t="str">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E33" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN1"] = "Manhattan";</v>
+      </c>
+      <c r="G33" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN1"] = "1";</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="B34" t="s">
+        <v>384</v>
+      </c>
+      <c r="C34" t="str">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E34" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN2"] = "Manhattan";</v>
+      </c>
+      <c r="G34" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN2"] = "2";</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="B35" t="s">
+        <v>384</v>
+      </c>
+      <c r="C35" t="str">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E35" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN3"] = "Manhattan";</v>
+      </c>
+      <c r="G35" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN3"] = "3";</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="B36" t="s">
+        <v>384</v>
+      </c>
+      <c r="C36" t="str">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E36" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN4"] = "Manhattan";</v>
+      </c>
+      <c r="G36" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN4"] = "4";</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B37" t="s">
+        <v>384</v>
+      </c>
+      <c r="C37" t="str">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E37" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN5"] = "Manhattan";</v>
+      </c>
+      <c r="G37" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN5"] = "5";</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="B38" t="s">
+        <v>384</v>
+      </c>
+      <c r="C38" t="str">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="E38" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN6"] = "Manhattan";</v>
+      </c>
+      <c r="G38" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN6"] = "6";</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B39" t="s">
+        <v>384</v>
+      </c>
+      <c r="C39" t="str">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E39" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN7"] = "Manhattan";</v>
+      </c>
+      <c r="G39" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN7"] = "7";</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="B40" t="s">
+        <v>384</v>
+      </c>
+      <c r="C40" t="str">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="E40" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN8"] = "Manhattan";</v>
+      </c>
+      <c r="G40" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN8"] = "8";</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B41" t="s">
+        <v>384</v>
+      </c>
+      <c r="C41" t="str">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="E41" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN9"] = "Manhattan";</v>
+      </c>
+      <c r="G41" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN9"] = "9";</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="B42" t="s">
+        <v>384</v>
+      </c>
+      <c r="C42" t="str">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="E42" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN10"] = "Manhattan";</v>
+      </c>
+      <c r="G42" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN10"] = "10";</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="B43" t="s">
+        <v>384</v>
+      </c>
+      <c r="C43" t="str">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="E43" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN11"] = "Manhattan";</v>
+      </c>
+      <c r="G43" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN11"] = "11";</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="B44" t="s">
+        <v>384</v>
+      </c>
+      <c r="C44" t="str">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="E44" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["MN12"] = "Manhattan";</v>
+      </c>
+      <c r="G44" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["MN12"] = "12";</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B45" t="s">
+        <v>383</v>
+      </c>
+      <c r="C45" t="str">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E45" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN1"] = "Queens";</v>
+      </c>
+      <c r="G45" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN1"] = "1";</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="B46" t="s">
+        <v>383</v>
+      </c>
+      <c r="C46" t="str">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E46" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN2"] = "Queens";</v>
+      </c>
+      <c r="G46" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN2"] = "2";</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="B47" t="s">
+        <v>383</v>
+      </c>
+      <c r="C47" t="str">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E47" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN3"] = "Queens";</v>
+      </c>
+      <c r="G47" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN3"] = "3";</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B48" t="s">
+        <v>383</v>
+      </c>
+      <c r="C48" t="str">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E48" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN4"] = "Queens";</v>
+      </c>
+      <c r="G48" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN4"] = "4";</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="B49" t="s">
+        <v>383</v>
+      </c>
+      <c r="C49" t="str">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E49" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN5"] = "Queens";</v>
+      </c>
+      <c r="G49" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN5"] = "5";</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="B50" t="s">
+        <v>383</v>
+      </c>
+      <c r="C50" t="str">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="E50" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN6"] = "Queens";</v>
+      </c>
+      <c r="G50" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN6"] = "6";</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B51" t="s">
+        <v>383</v>
+      </c>
+      <c r="C51" t="str">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E51" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN7"] = "Queens";</v>
+      </c>
+      <c r="G51" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN7"] = "7";</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="B52" t="s">
+        <v>383</v>
+      </c>
+      <c r="C52" t="str">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="E52" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN8"] = "Queens";</v>
+      </c>
+      <c r="G52" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN8"] = "8";</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B53" t="s">
+        <v>383</v>
+      </c>
+      <c r="C53" t="str">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="E53" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN9"] = "Queens";</v>
+      </c>
+      <c r="G53" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN9"] = "9";</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="B54" t="s">
+        <v>383</v>
+      </c>
+      <c r="C54" t="str">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="E54" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN10"] = "Queens";</v>
+      </c>
+      <c r="G54" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN10"] = "10";</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="B55" t="s">
+        <v>383</v>
+      </c>
+      <c r="C55" t="str">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="E55" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN11"] = "Queens";</v>
+      </c>
+      <c r="G55" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN11"] = "11";</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B56" t="s">
+        <v>383</v>
+      </c>
+      <c r="C56" t="str">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="E56" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN12"] = "Queens";</v>
+      </c>
+      <c r="G56" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN12"] = "12";</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="B57" t="s">
+        <v>383</v>
+      </c>
+      <c r="C57" t="str">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="E57" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN13"] = "Queens";</v>
+      </c>
+      <c r="G57" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN13"] = "13";</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="B58" t="s">
+        <v>383</v>
+      </c>
+      <c r="C58" t="str">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="E58" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["QN14"] = "Queens";</v>
+      </c>
+      <c r="G58" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["QN14"] = "14";</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="B59" t="s">
+        <v>382</v>
+      </c>
+      <c r="C59" t="str">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E59" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["SI1"] = "Staten Island";</v>
+      </c>
+      <c r="G59" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["SI1"] = "1";</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="B60" t="s">
+        <v>382</v>
+      </c>
+      <c r="C60" t="str">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E60" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["SI2"] = "Staten Island";</v>
+      </c>
+      <c r="G60" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["SI2"] = "2";</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="B61" t="s">
+        <v>382</v>
+      </c>
+      <c r="C61" t="str">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E61" t="str">
+        <f t="shared" si="1"/>
+        <v>boros["SI3"] = "Staten Island";</v>
+      </c>
+      <c r="G61" t="str">
+        <f t="shared" si="2"/>
+        <v>boards["SI3"] = "3";</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A62" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Some edits for FY27
</commit_message>
<xml_diff>
--- a/public/csvdata/variablenamelookups.xlsx
+++ b/public/csvdata/variablenamelookups.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidhochbaum/ae-cd-needs-statements-generator/public/csvdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C15C67-28CC-674E-9C4C-A3790303780D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4928F9BB-6116-764B-82AE-D76C31CD5A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="56460" yWindow="-11200" windowWidth="26240" windowHeight="32260" activeTab="3" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
+    <workbookView xWindow="56460" yWindow="-11080" windowWidth="26240" windowHeight="32260" activeTab="1" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Statements" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="397">
   <si>
     <t>Response ID</t>
   </si>
@@ -1228,6 +1228,12 @@
   </si>
   <si>
     <t>borough</t>
+  </si>
+  <si>
+    <t>Change History</t>
+  </si>
+  <si>
+    <t>Currently Logged In User</t>
   </si>
 </sst>
 </file>
@@ -3414,7 +3420,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6F5E8B0-77B9-4E4F-8066-17FC89ECA64A}">
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="130" bestFit="1" customWidth="1"/>
@@ -3864,6 +3870,16 @@
       </c>
       <c r="B73" t="s">
         <v>222</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>396</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added formulas to variablenamelookups
</commit_message>
<xml_diff>
--- a/public/csvdata/variablenamelookups.xlsx
+++ b/public/csvdata/variablenamelookups.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidhochbaum/ae-cd-needs-statements-generator/public/csvdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4928F9BB-6116-764B-82AE-D76C31CD5A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13354A84-D897-9044-AE73-07CA6BC966F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="56460" yWindow="-11080" windowWidth="26240" windowHeight="32260" activeTab="1" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
+    <workbookView xWindow="56460" yWindow="-11080" windowWidth="26240" windowHeight="31900" activeTab="1" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Statements" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="399">
   <si>
     <t>Response ID</t>
   </si>
@@ -1234,6 +1234,12 @@
   </si>
   <si>
     <t>Currently Logged In User</t>
+  </si>
+  <si>
+    <t>VLOOKUP(AC3,'[variablenamelookups.xlsx]Agency Acronyms'!$A:$B,2,0)</t>
+  </si>
+  <si>
+    <t>VLOOKUP(Y3,'[variablenamelookups.xlsx]boro&amp;board'!$A:$D,2,0)</t>
   </si>
 </sst>
 </file>
@@ -3420,33 +3426,39 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6F5E8B0-77B9-4E4F-8066-17FC89ECA64A}">
-  <dimension ref="A1:B75"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="130" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C1" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C4" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -3454,57 +3466,57 @@
         <v>101</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Updated with FY27 Agency Responses
</commit_message>
<xml_diff>
--- a/public/csvdata/variablenamelookups.xlsx
+++ b/public/csvdata/variablenamelookups.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidhochbaum/ae-cd-needs-statements-generator/public/csvdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13354A84-D897-9044-AE73-07CA6BC966F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35FDF8F4-A7B1-CF42-8434-6ED7DFD0165A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="56460" yWindow="-11080" windowWidth="26240" windowHeight="31900" activeTab="1" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
+    <workbookView xWindow="56460" yWindow="-11100" windowWidth="26240" windowHeight="31900" activeTab="1" xr2:uid="{B1E9EA43-BE9B-DF4F-AE25-49A3B01FF3EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Statements" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="399">
   <si>
     <t>Response ID</t>
   </si>
@@ -3852,9 +3852,15 @@
       <c r="A68" t="s">
         <v>205</v>
       </c>
+      <c r="B68" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
+        <v>206</v>
+      </c>
+      <c r="B69" t="s">
         <v>206</v>
       </c>
     </row>

</xml_diff>